<commit_message>
Cap nhat file excel moi
</commit_message>
<xml_diff>
--- a/TEST CASE/Test Cases Template.xlsx
+++ b/TEST CASE/Test Cases Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19890" windowHeight="7095"/>
+    <workbookView windowWidth="19890" windowHeight="7695"/>
   </bookViews>
   <sheets>
     <sheet name="Danh Sách Test_Case" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,16 @@
     <sheet name="TC_04" sheetId="5" r:id="rId5"/>
     <sheet name="TC_05" sheetId="6" r:id="rId6"/>
     <sheet name="TC_06" sheetId="7" r:id="rId7"/>
+    <sheet name="TC_07" sheetId="8" r:id="rId8"/>
+    <sheet name="TC_08" sheetId="9" r:id="rId9"/>
+    <sheet name="TC_09" sheetId="10" r:id="rId10"/>
+    <sheet name="TC_10" sheetId="11" r:id="rId11"/>
+    <sheet name="TC_11" sheetId="12" r:id="rId12"/>
+    <sheet name="TC_12" sheetId="13" r:id="rId13"/>
+    <sheet name="TC_13" sheetId="14" r:id="rId14"/>
+    <sheet name="TC_14" sheetId="15" r:id="rId15"/>
+    <sheet name="TC_15" sheetId="16" r:id="rId16"/>
+    <sheet name="TC_16" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="132">
   <si>
     <t>NOT TEST YET</t>
   </si>
@@ -188,6 +198,219 @@
     <t>TC_06!A1</t>
   </si>
   <si>
+    <t>TC_7</t>
+  </si>
+  <si>
+    <t>Quản lý bảng Sudoku</t>
+  </si>
+  <si>
+    <t>Kiểm tra khởi tạo bảng Sudoku 9x9 không hợp lệ</t>
+  </si>
+  <si>
+    <t>Truyền initial_grid hoặc solution_grid không đủ, vượt quá kích thước 9x9 ví dụ ma trận 8x8 hoặc 10x9</t>
+  </si>
+  <si>
+    <t>Hệ thống kiểm tra ra lỗi valueError ("Lưới ban đầu phải là ma trận 9x9)</t>
+  </si>
+  <si>
+    <t>Bắt được ngoại lệ ValueError chính xác như thiết kế</t>
+  </si>
+  <si>
+    <t>TC_07!A1</t>
+  </si>
+  <si>
+    <t>TC_8</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhập nước đi hợp lệ</t>
+  </si>
+  <si>
+    <t>Gọi set_value(row, col, val) với giá trị đúng với solition_grid</t>
+  </si>
+  <si>
+    <t>current_grid cập nhật giá trị mới, hàm trả về True</t>
+  </si>
+  <si>
+    <t>Điếm số  thành công, trả về True</t>
+  </si>
+  <si>
+    <t>TC_08!A1</t>
+  </si>
+  <si>
+    <t>TC_9</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhập nước đi sai ô cố định</t>
+  </si>
+  <si>
+    <t>Gọi set_value vào ô có initial_grid khác 0</t>
+  </si>
+  <si>
+    <t>Kiếm ra lỗi ValueError("Không thể chỉnh sửa ô cố định...")</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi không cho sửa ô cố định</t>
+  </si>
+  <si>
+    <t>TC_09!A1</t>
+  </si>
+  <si>
+    <t>TC_10</t>
+  </si>
+  <si>
+    <t>Kiểm tra điều kiện thắng game</t>
+  </si>
+  <si>
+    <t>Điền đúng toàn bộ các ô trùng khớp solution_grid</t>
+  </si>
+  <si>
+    <t>check_win_condition()   trả về True</t>
+  </si>
+  <si>
+    <t>Trả về True, hoàn thành game</t>
+  </si>
+  <si>
+    <t>TC_10!A1</t>
+  </si>
+  <si>
+    <t>TC_11</t>
+  </si>
+  <si>
+    <t>Quản lý đếm giờ</t>
+  </si>
+  <si>
+    <t>Kiểm tra phạt thời gian và đếm ngược</t>
+  </si>
+  <si>
+    <t>Chạy time ở chế độ countdown, gọi add_penalty(10)</t>
+  </si>
+  <si>
+    <t>Thời gian còn lại giảm đi 10 giây</t>
+  </si>
+  <si>
+    <t>Định dạng thời gian MM:SS hiển thị trừ chính xác</t>
+  </si>
+  <si>
+    <t>TC_11!A1</t>
+  </si>
+  <si>
+    <t>TC_12</t>
+  </si>
+  <si>
+    <t>Tính điểm</t>
+  </si>
+  <si>
+    <t>Kiểm tra cộng, trừ điểm và phạt</t>
+  </si>
+  <si>
+    <t>Gọi on_correct_move() và on_incorrect_move()</t>
+  </si>
+  <si>
+    <t>correct cộng 10đ; incorrect trừ 5đ và tăng số lỗi (errors) lên 1</t>
+  </si>
+  <si>
+    <t>Điểm số và số lỗi cập nhật chính xác</t>
+  </si>
+  <si>
+    <t>TC_12!A1</t>
+  </si>
+  <si>
+    <t>TC_13</t>
+  </si>
+  <si>
+    <t>Kiểm tra số trùng hàng</t>
+  </si>
+  <si>
+    <t>Nhập số đã xuất hiện trong cùng hàng</t>
+  </si>
+  <si>
+    <t>Trả về False</t>
+  </si>
+  <si>
+    <t>TC_13!A1</t>
+  </si>
+  <si>
+    <t>TC_14</t>
+  </si>
+  <si>
+    <t>Kiêm tra số trùng cột</t>
+  </si>
+  <si>
+    <t>Nhập số đã xuất hiện trong cùng cột</t>
+  </si>
+  <si>
+    <t>Trả vè False</t>
+  </si>
+  <si>
+    <t>TC_14!A1</t>
+  </si>
+  <si>
+    <t>TC_15</t>
+  </si>
+  <si>
+    <t>Kiểm tra số trùng ô 3x3</t>
+  </si>
+  <si>
+    <t>TC_15!A1</t>
+  </si>
+  <si>
+    <t>TC_16</t>
+  </si>
+  <si>
+    <t>Kiểm tra giá trị ngoài 0-9</t>
+  </si>
+  <si>
+    <t>TC_16!A1</t>
+  </si>
+  <si>
+    <t>TC_17</t>
+  </si>
+  <si>
+    <t>Kiểm tra toạ độ ngoài phạm vi</t>
+  </si>
+  <si>
+    <t>Phát sinh IndexError</t>
+  </si>
+  <si>
+    <t>TC_18</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhập số sai đáp án</t>
+  </si>
+  <si>
+    <t>Kiểm tra khi nhập số không bị trùng hàng/cột/khối nhưng không khớp với lời giải (solution_grid)</t>
+  </si>
+  <si>
+    <t>Gọi set_value(row, col, val) với val != solution_grid[row][col]</t>
+  </si>
+  <si>
+    <t>Trả về False (không khớp đáp án)</t>
+  </si>
+  <si>
+    <t>TC_19</t>
+  </si>
+  <si>
+    <t>Tính phần trăm tiến độ completion</t>
+  </si>
+  <si>
+    <t>Gọi get_progress() hoặc get_correct_progress()</t>
+  </si>
+  <si>
+    <t>Trả về tỉ lệ % chính xác (ví dụ điền 81/81 ô thì 100%</t>
+  </si>
+  <si>
+    <t>TC_20</t>
+  </si>
+  <si>
+    <t>Tính năng tạm dừng/tiếp tục đồng hồ</t>
+  </si>
+  <si>
+    <t>Gọi pause(), chờ 2 giây và sao đó gọi resume()</t>
+  </si>
+  <si>
+    <t>Thời gian trôi qua không cộng thêm 2 giây trong luc tạm dừng</t>
+  </si>
+  <si>
     <t>TC_01</t>
   </si>
   <si>
@@ -210,6 +433,12 @@
   </si>
   <si>
     <t>TC_06</t>
+  </si>
+  <si>
+    <t>TC_07</t>
+  </si>
+  <si>
+    <t>TC_08</t>
   </si>
 </sst>
 </file>
@@ -222,7 +451,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,13 +463,6 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -804,150 +1026,150 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -968,29 +1190,37 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Chung" xfId="0" builtinId="0"/>
@@ -1045,7 +1275,7 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left/>
         <right style="thin">
@@ -1060,7 +1290,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1077,7 +1307,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1094,7 +1324,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1111,7 +1341,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1128,7 +1358,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1145,7 +1375,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1162,7 +1392,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1179,7 +1409,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1196,7 +1426,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -1536,9 +1766,95 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="07"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="4352925" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="08-11-12"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="4019550" cy="704850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="B2:K8" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:K8" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="B2:K24" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:K24" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="10">
     <tableColumn id="1" name="No" dataDxfId="0"/>
     <tableColumn id="2" name="Name/Screen" dataDxfId="1"/>
@@ -1813,16 +2129,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:AL8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="7"/>
+  <dimension ref="B1:AL25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.1047619047619" style="1" customWidth="1"/>
-    <col min="2" max="2" width="5.66666666666667" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.3428571428571" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.71428571428571" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.4571428571429" style="1" customWidth="1"/>
     <col min="4" max="5" width="26.2190476190476" style="2" customWidth="1"/>
     <col min="6" max="6" width="27.7904761904762" style="2" customWidth="1"/>
-    <col min="7" max="7" width="36.4857142857143" style="1" customWidth="1"/>
-    <col min="8" max="9" width="26.2190476190476" style="1" customWidth="1"/>
+    <col min="7" max="7" width="51.152380952381" style="1" customWidth="1"/>
+    <col min="8" max="8" width="70.4571428571429" style="1" customWidth="1"/>
+    <col min="9" max="9" width="26.2190476190476" style="1" customWidth="1"/>
     <col min="10" max="10" width="17.7809523809524" style="1" customWidth="1"/>
     <col min="11" max="11" width="20" style="1" customWidth="1"/>
     <col min="12" max="12" width="19.4380952380952" style="1" customWidth="1"/>
@@ -2024,16 +2341,16 @@
       <c r="B8" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="14" t="s">
         <v>48</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -2044,12 +2361,391 @@
       <c r="J8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="14" t="s">
+      <c r="K8" s="15" t="s">
         <v>50</v>
       </c>
     </row>
+    <row r="9" ht="60" spans="2:38">
+      <c r="B9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" ht="45" spans="2:38">
+      <c r="B10" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" ht="30" spans="2:38">
+      <c r="B11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" ht="30" spans="2:38">
+      <c r="B12" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" ht="45" spans="2:38">
+      <c r="B13" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" ht="30" spans="2:38">
+      <c r="B14" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" ht="30" spans="2:38">
+      <c r="B15" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" ht="30" spans="2:38">
+      <c r="B16" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11">
+      <c r="B17" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11">
+      <c r="B18" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11">
+      <c r="B19" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K19" s="10"/>
+    </row>
+    <row r="20" ht="60" spans="2:11">
+      <c r="B20" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K20" s="10"/>
+    </row>
+    <row r="21" ht="30" spans="2:11">
+      <c r="B21" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K21" s="10"/>
+    </row>
+    <row r="22" ht="45" spans="2:11">
+      <c r="B22" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K22" s="10"/>
+    </row>
+    <row r="23" spans="2:11">
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K23" s="10"/>
+    </row>
+    <row r="24" spans="2:11">
+      <c r="B24" s="7"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="10"/>
+    </row>
+    <row r="25" spans="2:11">
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J3:J8">
+  <conditionalFormatting sqref="J3:J24">
     <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
       <formula>$AL$5</formula>
     </cfRule>
@@ -2058,7 +2754,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J24">
       <formula1>$AL$1:$AL$5</formula1>
     </dataValidation>
   </dataValidations>
@@ -2069,12 +2765,110 @@
     <hyperlink ref="K6" location="TC_04!A1" display="TC_04!A1"/>
     <hyperlink ref="K7" location="TC_05!A1" display="TC_05!A1"/>
     <hyperlink ref="K8" location="TC_06!A1" display="TC_06!A1"/>
+    <hyperlink ref="K9" location="TC_07!A1" display="TC_07!A1"/>
+    <hyperlink ref="K10" location="TC_08!A1" display="TC_08!A1"/>
+    <hyperlink ref="K11" location="TC_09!A1" display="TC_09!A1"/>
+    <hyperlink ref="K12" location="TC_10!A1" display="TC_10!A1"/>
+    <hyperlink ref="K13" location="TC_11!A1" display="TC_11!A1"/>
+    <hyperlink ref="K17" location="TC_15!A1" display="TC_15!A1"/>
+    <hyperlink ref="K18" location="TC_16!A1" display="TC_16!A1"/>
+    <hyperlink ref="K14" location="TC_12!A1" display="TC_12!A1"/>
+    <hyperlink ref="K15" location="TC_13!A1" display="TC_13!A1"/>
+    <hyperlink ref="K16" location="TC_14!A1" display="TC_14!A1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -2086,17 +2880,17 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>51</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="2:2">
       <c r="B3" t="s">
-        <v>52</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" t="s">
-        <v>53</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2114,17 +2908,17 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="2:2">
       <c r="B3" t="s">
-        <v>52</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" t="s">
-        <v>53</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2142,17 +2936,17 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>55</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="2:2">
       <c r="B3" t="s">
-        <v>52</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" t="s">
-        <v>53</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2170,7 +2964,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>56</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2188,7 +2982,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>57</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2206,7 +3000,43 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>58</v>
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
up date test case
</commit_message>
<xml_diff>
--- a/TEST CASE/Test Cases Template.xlsx
+++ b/TEST CASE/Test Cases Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19890" windowHeight="7695"/>
+    <workbookView windowWidth="20490" windowHeight="7095"/>
   </bookViews>
   <sheets>
     <sheet name="Danh Sách Test_Case" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,22 @@
     <sheet name="TC_14" sheetId="15" r:id="rId15"/>
     <sheet name="TC_15" sheetId="16" r:id="rId16"/>
     <sheet name="TC_16" sheetId="17" r:id="rId17"/>
+    <sheet name="TC_17" sheetId="18" r:id="rId18"/>
+    <sheet name="TC_18" sheetId="19" r:id="rId19"/>
+    <sheet name="TC_19" sheetId="20" r:id="rId20"/>
+    <sheet name="TC_20" sheetId="21" r:id="rId21"/>
+    <sheet name="TC_21" sheetId="22" r:id="rId22"/>
+    <sheet name="TC_22" sheetId="23" r:id="rId23"/>
+    <sheet name="TC_23" sheetId="24" r:id="rId24"/>
+    <sheet name="TC_24" sheetId="25" r:id="rId25"/>
+    <sheet name="TC_25" sheetId="26" r:id="rId26"/>
+    <sheet name="TC_26" sheetId="27" r:id="rId27"/>
+    <sheet name="TC_27" sheetId="28" r:id="rId28"/>
+    <sheet name="TC_28" sheetId="29" r:id="rId29"/>
+    <sheet name="TC_29" sheetId="30" r:id="rId30"/>
+    <sheet name="TC_30" sheetId="31" r:id="rId31"/>
+    <sheet name="TC_31" sheetId="32" r:id="rId32"/>
+    <sheet name="Bảo vệ trang tính33" sheetId="33" r:id="rId33"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="233">
   <si>
     <t>NOT TEST YET</t>
   </si>
@@ -93,7 +109,7 @@
     <t>Nhập 1</t>
   </si>
   <si>
-    <t>Tạo Sudoku dễ và in lời giải</t>
+    <t>Tạo Sudoku Dễ (xoá 35 ô) và in lời giải</t>
   </si>
   <si>
     <t>In đúng đề và lời giải phù hợp</t>
@@ -117,6 +133,9 @@
     <t>Nhập 2</t>
   </si>
   <si>
+    <t>Tạo Sudoku Vừa (xoá 45 ô) và in lời giải</t>
+  </si>
+  <si>
     <t>TC_02!A1</t>
   </si>
   <si>
@@ -129,6 +148,9 @@
     <t>Nhập 3</t>
   </si>
   <si>
+    <t>Tạo Sudoku Khó (xoá 55 ô) và in lời giải</t>
+  </si>
+  <si>
     <t>TC_03!A1</t>
   </si>
   <si>
@@ -162,10 +184,25 @@
     <t>Thuật toán sinh đề</t>
   </si>
   <si>
+    <t>Kiểm tra tính hợp lệ của hàm valid()</t>
+  </si>
+  <si>
+    <t>Gọi valid(broad, r, c, n) khi giá trị n đã xuất hiện trong hàng/cột/khối 3x3</t>
+  </si>
+  <si>
+    <t>Trả về False</t>
+  </si>
+  <si>
+    <t>Trả về False chính xác</t>
+  </si>
+  <si>
+    <t>TC_6</t>
+  </si>
+  <si>
     <t>Kiểm tra tính hợp lệ đề bài</t>
   </si>
   <si>
-    <t xml:space="preserve">Chạy sinh đề ngẫu nhiên </t>
+    <t>Gọi generate_sudoku("de") hoặc generate ("kho")</t>
   </si>
   <si>
     <t>Các số không bị trùng hàng/cột/khối</t>
@@ -177,7 +214,7 @@
     <t>TC_05!A1</t>
   </si>
   <si>
-    <t>TC_6</t>
+    <t>TC_7</t>
   </si>
   <si>
     <t>Thuật toán giải</t>
@@ -198,217 +235,496 @@
     <t>TC_06!A1</t>
   </si>
   <si>
-    <t>TC_7</t>
+    <t>TC_8</t>
+  </si>
+  <si>
+    <t>Kiểm tra giải đề với bàn cờ không có lời giải</t>
+  </si>
+  <si>
+    <t>Truyền bàn cờ bị xung đột số vào hàm backtracking(broad)</t>
+  </si>
+  <si>
+    <t>Hàm trả về False (không tìm thấy lời giải</t>
+  </si>
+  <si>
+    <t>Trả về False đúng xử lý</t>
+  </si>
+  <si>
+    <t>TC_9</t>
+  </si>
+  <si>
+    <t>Logic Sudoku (SudokuBoard)</t>
+  </si>
+  <si>
+    <t>Kiểm tra khởi tạo bảng Sudoku 9x9 không hợp lệ</t>
+  </si>
+  <si>
+    <t>Truyền initial_grid hoặc solution_grid không đủ, vượt quá kích thước 9x9 ví dụ ma trận 8x8 hoặc 10x9</t>
+  </si>
+  <si>
+    <t>Hệ thống kiểm tra ra lỗi valueError ("Lưới ban đầu phải là ma trận 9x9)</t>
+  </si>
+  <si>
+    <t>Bắt được ngoại lệ ValueError chính xác như thiết kế</t>
+  </si>
+  <si>
+    <t>TC_07!A1</t>
+  </si>
+  <si>
+    <t>TC_10</t>
+  </si>
+  <si>
+    <t>Kiểm tra quy tắc đặt số hợp lệ và trùng hàng/cột/khối 3x3</t>
+  </si>
+  <si>
+    <t>Gọi is_valid_sudoku_rule (row, col, value) với số bị trùng trong cùng hàng hoặc cột</t>
+  </si>
+  <si>
+    <t>Trả về False khi trùng số, trả về True khi vị trí đặt hợp lệ</t>
+  </si>
+  <si>
+    <t>Trả về kết quả kiểm tra luật đúng</t>
+  </si>
+  <si>
+    <t>TC_08!A1</t>
+  </si>
+  <si>
+    <t>TC_11</t>
+  </si>
+  <si>
+    <t>Kiểm tra thao tác ghi đè ô cố định ban đầu</t>
+  </si>
+  <si>
+    <t>Gọi set_value(row, col, val) tại vị trí ô ban đầu initial_grid khác 0</t>
+  </si>
+  <si>
+    <t>Quăng ngoại lệ ValueError("Không thể chỉnh sửa ô cố định...")</t>
+  </si>
+  <si>
+    <t>Chặn chỉnh sửa ô ban đầu thành công</t>
+  </si>
+  <si>
+    <t>TC_09!A1</t>
+  </si>
+  <si>
+    <t>TC_12</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính toán tỷ lệ tiến độ hoàn thành (get_progress)</t>
+  </si>
+  <si>
+    <t>Đã  điền 40 ô trên tổng 81 ô</t>
+  </si>
+  <si>
+    <t>Trả về tỷ lệ phần trăm khoản 49.38%</t>
+  </si>
+  <si>
+    <t>Tính đúng tỷ lệ phần trăm ô đã điền</t>
+  </si>
+  <si>
+    <t>TC_10!A1</t>
+  </si>
+  <si>
+    <t>TC_13</t>
+  </si>
+  <si>
+    <t>Bộ đếm thời gian(SudokuTimer)</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính năng tạm dừng (pause) và tiếp tục (resume)</t>
+  </si>
+  <si>
+    <t>Gọi start(), chờ 3 giây, gọi pause(), chờ 2 giây rồi gọi get_elapsed_time()</t>
+  </si>
+  <si>
+    <t>Thời gian trôi qua dừng lại ở 3 giây, không tính 2 giây trong lúc pause</t>
+  </si>
+  <si>
+    <t>Điếm thời gian chính xác theo trạng  thái</t>
+  </si>
+  <si>
+    <t>TC_11!A1</t>
+  </si>
+  <si>
+    <t>TC_14</t>
+  </si>
+  <si>
+    <t>Tính điểm(SudokuScoring)</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính điểm khi điền đúng và bị trừ điểm khi điền sai</t>
+  </si>
+  <si>
+    <t>Gọi on_correct_move() 2 lần, sau đó gọi on_incorrect_move() 1 lần</t>
+  </si>
+  <si>
+    <t>Tổng  điểm thu được là 10 x 2 - 5 = 15 điểm, số lỗi errors = 1</t>
+  </si>
+  <si>
+    <t>Tính tổng điểm và ghi nhận số lỗi chính xác</t>
+  </si>
+  <si>
+    <t>TC_12!A1</t>
+  </si>
+  <si>
+    <t>TC_15</t>
   </si>
   <si>
     <t>Quản lý bảng Sudoku</t>
   </si>
   <si>
-    <t>Kiểm tra khởi tạo bảng Sudoku 9x9 không hợp lệ</t>
-  </si>
-  <si>
-    <t>Truyền initial_grid hoặc solution_grid không đủ, vượt quá kích thước 9x9 ví dụ ma trận 8x8 hoặc 10x9</t>
-  </si>
-  <si>
-    <t>Hệ thống kiểm tra ra lỗi valueError ("Lưới ban đầu phải là ma trận 9x9)</t>
-  </si>
-  <si>
-    <t>Bắt được ngoại lệ ValueError chính xác như thiết kế</t>
-  </si>
-  <si>
-    <t>TC_07!A1</t>
-  </si>
-  <si>
-    <t>TC_8</t>
-  </si>
-  <si>
-    <t>Kiểm tra nhập nước đi hợp lệ</t>
-  </si>
-  <si>
-    <t>Gọi set_value(row, col, val) với giá trị đúng với solition_grid</t>
-  </si>
-  <si>
-    <t>current_grid cập nhật giá trị mới, hàm trả về True</t>
-  </si>
-  <si>
-    <t>Điếm số  thành công, trả về True</t>
-  </si>
-  <si>
-    <t>TC_08!A1</t>
-  </si>
-  <si>
-    <t>TC_9</t>
-  </si>
-  <si>
-    <t>Kiểm tra nhập nước đi sai ô cố định</t>
-  </si>
-  <si>
-    <t>Gọi set_value vào ô có initial_grid khác 0</t>
-  </si>
-  <si>
-    <t>Kiếm ra lỗi ValueError("Không thể chỉnh sửa ô cố định...")</t>
-  </si>
-  <si>
-    <t>Hệ thống báo lỗi không cho sửa ô cố định</t>
-  </si>
-  <si>
-    <t>TC_09!A1</t>
-  </si>
-  <si>
-    <t>TC_10</t>
-  </si>
-  <si>
-    <t>Kiểm tra điều kiện thắng game</t>
-  </si>
-  <si>
-    <t>Điền đúng toàn bộ các ô trùng khớp solution_grid</t>
-  </si>
-  <si>
-    <t>check_win_condition()   trả về True</t>
-  </si>
-  <si>
-    <t>Trả về True, hoàn thành game</t>
-  </si>
-  <si>
-    <t>TC_10!A1</t>
-  </si>
-  <si>
-    <t>TC_11</t>
+    <t>Kiểm tra số trùng hàng</t>
+  </si>
+  <si>
+    <t>Gọi is_valid_sudoku_rule với giá trị đã xuất hiện trong cùng hàng</t>
+  </si>
+  <si>
+    <t>TC_13!A1</t>
+  </si>
+  <si>
+    <t>TC_16</t>
+  </si>
+  <si>
+    <t>Kiểm tra số trùng cột</t>
+  </si>
+  <si>
+    <t>Gọi is_valid_sudoku_rule với giá trị đã xuất hiện trong cùng cột</t>
+  </si>
+  <si>
+    <t>Trả vè False</t>
+  </si>
+  <si>
+    <t>TC_14!A1</t>
+  </si>
+  <si>
+    <t>TC_17</t>
+  </si>
+  <si>
+    <t>Kiểm tra số trùng ô 3x3</t>
+  </si>
+  <si>
+    <t>Gọi is_valid_sudoku_rule với giá trị đã xuất hiện trong cùng khối 3x3</t>
+  </si>
+  <si>
+    <t>TC_15!A1</t>
+  </si>
+  <si>
+    <t>TC_18</t>
+  </si>
+  <si>
+    <t>Kiểm tra giá trị nhập vào ngoài khoảng  0-9</t>
+  </si>
+  <si>
+    <t>Gọi is_valid_sudoku_rule với giá trị âm (vd: -1) hoặc lớn hơn 9 (vd: 10)</t>
+  </si>
+  <si>
+    <t>TC_16!A1</t>
+  </si>
+  <si>
+    <t>TC_19</t>
+  </si>
+  <si>
+    <t>Kiểm tra toạ độ ngoài phạm vi ma trận</t>
+  </si>
+  <si>
+    <t>Gọi hàm bất kì với row hoặc col &lt; 0 hoặc &gt; 8</t>
+  </si>
+  <si>
+    <t>Phát sinh lỗi IndexError</t>
+  </si>
+  <si>
+    <t>TC_19!A1</t>
+  </si>
+  <si>
+    <t>TC_20</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhập số sai đáp án (không trùng lặp nhưng sai giải pháp)</t>
+  </si>
+  <si>
+    <t>Gọi set_value(row, col, val) với val khác solution_grid[row][col]</t>
+  </si>
+  <si>
+    <t>Trả về False (không khớp đáp án)</t>
+  </si>
+  <si>
+    <t>TC_20!A1</t>
+  </si>
+  <si>
+    <t>TC_21</t>
+  </si>
+  <si>
+    <t>Quản lý tiến độ</t>
+  </si>
+  <si>
+    <t>Tính phần trăm tiến độ hoàn thành</t>
+  </si>
+  <si>
+    <t>Gọi get_progress() khi đã điền đúng toàn bộ 81 ô</t>
+  </si>
+  <si>
+    <t>Trả về tỉ lệ % chính xác (ví dụ điền 81/81 ô thì 100%</t>
+  </si>
+  <si>
+    <t>TC_21!A1</t>
+  </si>
+  <si>
+    <t>TC_22</t>
   </si>
   <si>
     <t>Quản lý đếm giờ</t>
   </si>
   <si>
-    <t>Kiểm tra phạt thời gian và đếm ngược</t>
-  </si>
-  <si>
-    <t>Chạy time ở chế độ countdown, gọi add_penalty(10)</t>
-  </si>
-  <si>
-    <t>Thời gian còn lại giảm đi 10 giây</t>
-  </si>
-  <si>
-    <t>Định dạng thời gian MM:SS hiển thị trừ chính xác</t>
-  </si>
-  <si>
-    <t>TC_11!A1</t>
-  </si>
-  <si>
-    <t>TC_12</t>
-  </si>
-  <si>
-    <t>Tính điểm</t>
-  </si>
-  <si>
-    <t>Kiểm tra cộng, trừ điểm và phạt</t>
-  </si>
-  <si>
-    <t>Gọi on_correct_move() và on_incorrect_move()</t>
-  </si>
-  <si>
-    <t>correct cộng 10đ; incorrect trừ 5đ và tăng số lỗi (errors) lên 1</t>
-  </si>
-  <si>
-    <t>Điểm số và số lỗi cập nhật chính xác</t>
-  </si>
-  <si>
-    <t>TC_12!A1</t>
-  </si>
-  <si>
-    <t>TC_13</t>
-  </si>
-  <si>
-    <t>Kiểm tra số trùng hàng</t>
-  </si>
-  <si>
-    <t>Nhập số đã xuất hiện trong cùng hàng</t>
-  </si>
-  <si>
-    <t>Trả về False</t>
-  </si>
-  <si>
-    <t>TC_13!A1</t>
-  </si>
-  <si>
-    <t>TC_14</t>
-  </si>
-  <si>
-    <t>Kiêm tra số trùng cột</t>
-  </si>
-  <si>
-    <t>Nhập số đã xuất hiện trong cùng cột</t>
-  </si>
-  <si>
-    <t>Trả vè False</t>
-  </si>
-  <si>
-    <t>TC_14!A1</t>
-  </si>
-  <si>
-    <t>TC_15</t>
-  </si>
-  <si>
-    <t>Kiểm tra số trùng ô 3x3</t>
-  </si>
-  <si>
-    <t>TC_15!A1</t>
-  </si>
-  <si>
-    <t>TC_16</t>
-  </si>
-  <si>
-    <t>Kiểm tra giá trị ngoài 0-9</t>
-  </si>
-  <si>
-    <t>TC_16!A1</t>
-  </si>
-  <si>
-    <t>TC_17</t>
-  </si>
-  <si>
-    <t>Kiểm tra toạ độ ngoài phạm vi</t>
-  </si>
-  <si>
-    <t>Phát sinh IndexError</t>
-  </si>
-  <si>
-    <t>TC_18</t>
-  </si>
-  <si>
-    <t>Kiểm tra nhập số sai đáp án</t>
-  </si>
-  <si>
-    <t>Kiểm tra khi nhập số không bị trùng hàng/cột/khối nhưng không khớp với lời giải (solution_grid)</t>
-  </si>
-  <si>
-    <t>Gọi set_value(row, col, val) với val != solution_grid[row][col]</t>
-  </si>
-  <si>
-    <t>Trả về False (không khớp đáp án)</t>
-  </si>
-  <si>
-    <t>TC_19</t>
-  </si>
-  <si>
-    <t>Tính phần trăm tiến độ completion</t>
-  </si>
-  <si>
-    <t>Gọi get_progress() hoặc get_correct_progress()</t>
-  </si>
-  <si>
-    <t>Trả về tỉ lệ % chính xác (ví dụ điền 81/81 ô thì 100%</t>
-  </si>
-  <si>
-    <t>TC_20</t>
-  </si>
-  <si>
     <t>Tính năng tạm dừng/tiếp tục đồng hồ</t>
   </si>
   <si>
     <t>Gọi pause(), chờ 2 giây và sao đó gọi resume()</t>
   </si>
   <si>
-    <t>Thời gian trôi qua không cộng thêm 2 giây trong luc tạm dừng</t>
+    <t>Thời gian trôi qua không cộng thêm 2 giây trong lúc tạm dừng</t>
+  </si>
+  <si>
+    <t>TC_22!A1</t>
+  </si>
+  <si>
+    <t>TC_23</t>
+  </si>
+  <si>
+    <t>Màn hình đăng nhập</t>
+  </si>
+  <si>
+    <t>Kiểm tra hiển thị đầy đủ các phần tử giao diện login.html</t>
+  </si>
+  <si>
+    <t>Mở trang login.html trên trình duyệt</t>
+  </si>
+  <si>
+    <t>Hiển thị đủ ô nhập Tên đăng nhập, Mật khẩu, Nút đăng nhập, checkbox Lưu mật khẩu và quên mật khẩu</t>
+  </si>
+  <si>
+    <t>Đã hiển thị đầy đủ giao diện</t>
+  </si>
+  <si>
+    <t>TC_24</t>
+  </si>
+  <si>
+    <t>Kiểm tra ẩn kí tự mật khẩu</t>
+  </si>
+  <si>
+    <t>Nhập chuỗi bất kỳ vào ô mật khẩu (ví dụ: 123456)</t>
+  </si>
+  <si>
+    <t>Các kí tự nhập vào hiển thị dạng dấu chấm đen/mặt định ẩn</t>
+  </si>
+  <si>
+    <t>Mật khẩu được ẩn đúng chuẩn type="password"</t>
+  </si>
+  <si>
+    <t>TC_25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiểm tra hành vi khi nhấn nút Đăng nhập mà để trống thông tin </t>
+  </si>
+  <si>
+    <t>Để trống ô Tên đăng nhập và Mật khẩu, nhấn nút Đăng nhập</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi và yêu cầu nhập thông tin (hiện tại form thiếu attribute required nên sẽ chưa chặn submit)</t>
+  </si>
+  <si>
+    <t>Form chưa validate dữ liệu trống</t>
+  </si>
+  <si>
+    <t>TC_26</t>
+  </si>
+  <si>
+    <t>Kết nối Client</t>
+  </si>
+  <si>
+    <t>Kiểm tra đăng ký tên người chơi qua Socket</t>
+  </si>
+  <si>
+    <t>Chạy Client.py và nhập tên: Bao Bao</t>
+  </si>
+  <si>
+    <t>Gửi chuỗi NAME|BaoBao, Sever phản hồi WELCOME</t>
+  </si>
+  <si>
+    <t>Kết nối thành công, nhận chào mừng</t>
+  </si>
+  <si>
+    <t>TC_26!A1</t>
+  </si>
+  <si>
+    <t>TC_27</t>
+  </si>
+  <si>
+    <t>Đăng nhập sever</t>
+  </si>
+  <si>
+    <t>Kiểm tra gửi message Đăng nhập dạng JSON</t>
+  </si>
+  <si>
+    <t>Gửi JSON {"type": "Đăng nhập", "playerId": "P1", "playerName": "BaoBao"}</t>
+  </si>
+  <si>
+    <t>Sever lưu danh sách playes và trả về Đăng nhập thành công</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công</t>
+  </si>
+  <si>
+    <t>TC_27!A1</t>
+  </si>
+  <si>
+    <t>TC_28</t>
+  </si>
+  <si>
+    <t>Tạo phòng</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính năng tạo phòng chơi mới</t>
+  </si>
+  <si>
+    <t>Gửi JSON {"type": "Tạo Phòng", "playerId": "P1"}</t>
+  </si>
+  <si>
+    <t>Sever tạo roomId ngẫu nhiên, cập nhật trạng thái "Đang Chờ"</t>
+  </si>
+  <si>
+    <t>Tạo phòng thành công</t>
+  </si>
+  <si>
+    <t>TC_28!A1</t>
+  </si>
+  <si>
+    <t>TC_29</t>
+  </si>
+  <si>
+    <t>Tham gia phòng</t>
+  </si>
+  <si>
+    <t>Kiểm tra người chơi thứ 2 vào phòng</t>
+  </si>
+  <si>
+    <t>Gửi JSON {"type": "Tham gia phòng", "roomID": "1234", "playerID": "BanhMi"}</t>
+  </si>
+  <si>
+    <t>Thêm P2 vào phòng, chuyển trạng thái phòng sang "Đang chơi" khi đủ 2 người</t>
+  </si>
+  <si>
+    <t>Đủ 2 người chơi, sẵn sàng ghép trận</t>
+  </si>
+  <si>
+    <t>TC_29!A1</t>
+  </si>
+  <si>
+    <t>TC_30</t>
+  </si>
+  <si>
+    <t>Xử lý lỗi phòng</t>
+  </si>
+  <si>
+    <t>Kiểm tra vào phòng không tồn tại</t>
+  </si>
+  <si>
+    <t>Gửi yêu cầu với roomId không  có trong hệ thống</t>
+  </si>
+  <si>
+    <t>Sever trả về phản hồi {"type": "Phòng không tồn tại"}</t>
+  </si>
+  <si>
+    <t>Báo lỗi phòng không tồn tại chính xác</t>
+  </si>
+  <si>
+    <t>TC_31</t>
+  </si>
+  <si>
+    <t>Bắt đầu trận đấu</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhận sự kiện bắt đầu bàn chơi từ Client</t>
+  </si>
+  <si>
+    <t>Client nhận message MATH_START từ Sever</t>
+  </si>
+  <si>
+    <t>Client in thông báo trận đấu bắt đầu, tên đối thủ và vẽ bàn cờ  Sudoku</t>
+  </si>
+  <si>
+    <t>Vẽ bàn cờ và hiển thị thông tin đối thủ đúng</t>
+  </si>
+  <si>
+    <t>TC_32</t>
+  </si>
+  <si>
+    <t>Quản lý lượt đi</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhận thông báo lượt chơi (TURN)</t>
+  </si>
+  <si>
+    <t>Sever gửi TURN|BaoBao|30|&lt;broad&gt;</t>
+  </si>
+  <si>
+    <t>Nếu đúng tên người chơi thì hiện ô nhập nước đi, ngược lại in "Đợi lượt đối thủ..."</t>
+  </si>
+  <si>
+    <t>Phân lượt đi chính xác</t>
+  </si>
+  <si>
+    <t>TC_33</t>
+  </si>
+  <si>
+    <t>Gửi nước đi</t>
+  </si>
+  <si>
+    <t>Kiểm tra định dạng nước đi gửi lên Sever</t>
+  </si>
+  <si>
+    <t>Nhập nước đi từ bàn phím: 0 1 5</t>
+  </si>
+  <si>
+    <t>Client  format thành chuỗi MOVE|0|1|5 và gửi qua socket</t>
+  </si>
+  <si>
+    <t>Gửi nước đi đúng định dạng</t>
+  </si>
+  <si>
+    <t>TC_34</t>
+  </si>
+  <si>
+    <t>Bắt lỗi nhập liệu</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhập nước đi sai định dạng ở Client</t>
+  </si>
+  <si>
+    <t>Nhập chuỗi không phải số (vd: abc hoặc 01)</t>
+  </si>
+  <si>
+    <t>Client  bắt lỗi ValueError và in thông báo yêu cầu nhập lại</t>
+  </si>
+  <si>
+    <t>Không bị crash app, báo lỗi nhập lại</t>
+  </si>
+  <si>
+    <t>TC_35</t>
+  </si>
+  <si>
+    <t>Ngắt kết nối</t>
+  </si>
+  <si>
+    <t>Kiểm tra nhận kết quả trận đấu (RESULT) hoặc ngắt kết nối</t>
+  </si>
+  <si>
+    <t>Sever gửi RESULT|BaoBao|Thắng hoặc đóng Socket</t>
+  </si>
+  <si>
+    <t>Client in kết quả thắng/ thua, dừng luồng nhận và đóng Socket an toàn</t>
+  </si>
+  <si>
+    <t>Đóng kết nối an toàn, hoàn thành bài test</t>
   </si>
   <si>
     <t>TC_01</t>
@@ -439,6 +755,9 @@
   </si>
   <si>
     <t>TC_08</t>
+  </si>
+  <si>
+    <t>TC-26</t>
   </si>
 </sst>
 </file>
@@ -1513,6 +1832,345 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="20"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="2143125" cy="666750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="21"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="4610100" cy="819150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="22"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="2686050" cy="3467100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="khởi tạo server tc_26"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="5172075" cy="428625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="27"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="5267325" cy="876300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Hình ảnh 3" descr="2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="1533525"/>
+          <a:ext cx="9363075" cy="1581150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Hình ảnh 2" descr="29"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="9363075" cy="2324100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="9363075" cy="1581150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -1852,9 +2510,52 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1" descr="19"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="390525"/>
+          <a:ext cx="8905875" cy="3019425"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="B2:K24" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:K24" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="B2:K37" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:K37" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="10">
     <tableColumn id="1" name="No" dataDxfId="0"/>
     <tableColumn id="2" name="Name/Screen" dataDxfId="1"/>
@@ -2129,7 +2830,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:AL25"/>
+  <dimension ref="B1:AL38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.1047619047619" style="1" customWidth="1"/>
@@ -2188,7 +2889,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="2:38">
+    <row r="3" ht="30" spans="2:38">
       <c r="B3" s="7" t="s">
         <v>12</v>
       </c>
@@ -2219,7 +2920,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:38">
+    <row r="4" ht="30" spans="2:38">
       <c r="B4" s="7" t="s">
         <v>21</v>
       </c>
@@ -2233,7 +2934,7 @@
         <v>23</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>17</v>
@@ -2244,27 +2945,27 @@
         <v>18</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AL4" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:38">
+    <row r="5" ht="30" spans="2:38">
       <c r="B5" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>17</v>
@@ -2275,30 +2976,30 @@
         <v>18</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AL5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" ht="90" spans="2:38">
       <c r="B6" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
@@ -2306,127 +3007,119 @@
         <v>18</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" ht="30" spans="2:38">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" ht="45" spans="2:38">
       <c r="B7" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
-      <c r="J7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>43</v>
-      </c>
+      <c r="J7" s="8"/>
+      <c r="K7" s="10"/>
     </row>
     <row r="8" ht="30" spans="2:38">
-      <c r="B8" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="13" t="s">
+      <c r="B8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="C8" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="9" t="s">
         <v>48</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
       <c r="J8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="15" t="s">
+      <c r="K8" s="10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="9" ht="60" spans="2:38">
-      <c r="B9" s="7" t="s">
+    <row r="9" ht="30" spans="2:38">
+      <c r="B9" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="14" t="s">
         <v>55</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
       <c r="J9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="K9" s="15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="10" ht="45" spans="2:38">
-      <c r="B10" s="7" t="s">
+    <row r="10" ht="30" spans="2:38">
+      <c r="B10" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="14" t="s">
         <v>61</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="15"/>
+    </row>
+    <row r="11" ht="60" spans="2:38">
+      <c r="B11" s="7" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="11" ht="30" spans="2:38">
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>65</v>
@@ -2443,18 +3136,18 @@
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
       <c r="J11" s="8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="12" ht="30" spans="2:38">
+    <row r="12" ht="60" spans="2:38">
       <c r="B12" s="7" t="s">
         <v>70</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>71</v>
@@ -2471,9 +3164,9 @@
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
       <c r="J12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K12" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" s="10" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2482,206 +3175,232 @@
         <v>76</v>
       </c>
       <c r="C13" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="E13" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="F13" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>81</v>
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K13" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" ht="45" spans="2:38">
+      <c r="B14" s="7" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="14" ht="30" spans="2:38">
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="F14" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>86</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>88</v>
       </c>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
       <c r="J14" s="8" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="K14" s="16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" ht="45" spans="2:38">
+      <c r="B15" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="15" ht="30" spans="2:38">
-      <c r="B15" s="7" t="s">
+      <c r="D15" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="E15" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9" t="s">
+      <c r="F15" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="G15" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
       <c r="J15" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K15" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K15" s="16" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="16" ht="30" spans="2:38">
+    <row r="16" ht="45" spans="2:38">
       <c r="B16" s="7" t="s">
         <v>95</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="9"/>
+      <c r="D16" s="9" t="s">
+        <v>97</v>
+      </c>
       <c r="E16" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G16" s="8"/>
+        <v>99</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>100</v>
+      </c>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K16" s="18" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="2:11">
+        <v>18</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" ht="45" spans="2:11">
       <c r="B17" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
+        <v>103</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>105</v>
+      </c>
       <c r="F17" s="9" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
       <c r="J17" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K17" s="16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="18" spans="2:11">
+        <v>18</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" ht="45" spans="2:11">
       <c r="B18" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
+      <c r="D18" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>109</v>
+      </c>
       <c r="F18" s="9" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
       <c r="J18" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K18" s="16" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="19" spans="2:11">
+        <v>18</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" ht="45" spans="2:11">
       <c r="B19" s="7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
+        <v>103</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>114</v>
+      </c>
       <c r="F19" s="9" t="s">
-        <v>108</v>
+        <v>43</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
       <c r="J19" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K19" s="10"/>
-    </row>
-    <row r="20" ht="60" spans="2:11">
+        <v>18</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" ht="45" spans="2:11">
       <c r="B20" s="7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
       <c r="J20" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K20" s="10"/>
+        <v>18</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="21" ht="30" spans="2:11">
       <c r="B21" s="7" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D21" s="9"/>
+        <v>103</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>121</v>
+      </c>
       <c r="E21" s="9" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
@@ -2689,21 +3408,25 @@
       <c r="J21" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K21" s="10"/>
+      <c r="K21" s="10" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="22" ht="45" spans="2:11">
       <c r="B22" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D22" s="9"/>
+        <v>103</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>126</v>
+      </c>
       <c r="E22" s="9" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
@@ -2711,41 +3434,407 @@
       <c r="J22" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K22" s="10"/>
-    </row>
-    <row r="23" spans="2:11">
-      <c r="B23" s="7"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
+      <c r="K22" s="16" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" ht="30" spans="2:11">
+      <c r="B23" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>134</v>
+      </c>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
       <c r="J23" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="10"/>
-    </row>
-    <row r="24" spans="2:11">
-      <c r="B24" s="7"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
+      <c r="K23" s="16" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" ht="45" spans="2:11">
+      <c r="B24" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>140</v>
+      </c>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="10"/>
-    </row>
-    <row r="25" spans="2:11">
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
+      <c r="J24" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K24" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" ht="60" spans="2:11">
+      <c r="B25" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K25" s="10"/>
+    </row>
+    <row r="26" ht="45" spans="2:11">
+      <c r="B26" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="10"/>
+    </row>
+    <row r="27" ht="60" spans="2:11">
+      <c r="B27" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K27" s="10"/>
+    </row>
+    <row r="28" ht="30" spans="2:11">
+      <c r="B28" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="29" ht="45" spans="2:11">
+      <c r="B29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K29" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="30" ht="30" spans="2:11">
+      <c r="B30" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K30" s="10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="31" ht="45" spans="2:11">
+      <c r="B31" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K31" s="10" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" ht="30" spans="2:11">
+      <c r="B32" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K32" s="10"/>
+    </row>
+    <row r="33" ht="45" spans="2:11">
+      <c r="B33" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K33" s="10"/>
+    </row>
+    <row r="34" ht="45" spans="2:11">
+      <c r="B34" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K34" s="10"/>
+    </row>
+    <row r="35" ht="30" spans="2:11">
+      <c r="B35" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="10"/>
+    </row>
+    <row r="36" ht="30" spans="2:11">
+      <c r="B36" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="10"/>
+    </row>
+    <row r="37" ht="45" spans="2:11">
+      <c r="B37" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="10"/>
+    </row>
+    <row r="38" spans="2:11">
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J3:J24">
+  <conditionalFormatting sqref="J3:J37">
     <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
       <formula>$AL$5</formula>
     </cfRule>
@@ -2754,7 +3843,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J37">
       <formula1>$AL$1:$AL$5</formula1>
     </dataValidation>
   </dataValidations>
@@ -2763,18 +3852,26 @@
     <hyperlink ref="K4" location="TC_02!A1" display="TC_02!A1"/>
     <hyperlink ref="K5" location="TC_03!A1" display="TC_03!A1"/>
     <hyperlink ref="K6" location="TC_04!A1" display="TC_04!A1"/>
-    <hyperlink ref="K7" location="TC_05!A1" display="TC_05!A1"/>
-    <hyperlink ref="K8" location="TC_06!A1" display="TC_06!A1"/>
-    <hyperlink ref="K9" location="TC_07!A1" display="TC_07!A1"/>
-    <hyperlink ref="K10" location="TC_08!A1" display="TC_08!A1"/>
-    <hyperlink ref="K11" location="TC_09!A1" display="TC_09!A1"/>
-    <hyperlink ref="K12" location="TC_10!A1" display="TC_10!A1"/>
-    <hyperlink ref="K13" location="TC_11!A1" display="TC_11!A1"/>
-    <hyperlink ref="K17" location="TC_15!A1" display="TC_15!A1"/>
-    <hyperlink ref="K18" location="TC_16!A1" display="TC_16!A1"/>
-    <hyperlink ref="K14" location="TC_12!A1" display="TC_12!A1"/>
-    <hyperlink ref="K15" location="TC_13!A1" display="TC_13!A1"/>
-    <hyperlink ref="K16" location="TC_14!A1" display="TC_14!A1"/>
+    <hyperlink ref="K8" location="TC_05!A1" display="TC_05!A1"/>
+    <hyperlink ref="K9" location="TC_06!A1" display="TC_06!A1"/>
+    <hyperlink ref="K11" location="TC_07!A1" display="TC_07!A1"/>
+    <hyperlink ref="K12" location="TC_08!A1" display="TC_08!A1"/>
+    <hyperlink ref="K13" location="TC_09!A1" display="TC_09!A1"/>
+    <hyperlink ref="K14" location="TC_10!A1" display="TC_10!A1"/>
+    <hyperlink ref="K15" location="TC_11!A1" display="TC_11!A1"/>
+    <hyperlink ref="K19" location="TC_15!A1" display="TC_15!A1"/>
+    <hyperlink ref="K20" location="TC_16!A1" display="TC_16!A1"/>
+    <hyperlink ref="K16" location="TC_12!A1" display="TC_12!A1"/>
+    <hyperlink ref="K17" location="TC_13!A1" display="TC_13!A1"/>
+    <hyperlink ref="K18" location="TC_14!A1" display="TC_14!A1"/>
+    <hyperlink ref="K29" location="TC_27!A1" display="TC_27!A1"/>
+    <hyperlink ref="K28" location="TC_26!A1" display="TC_26!A1"/>
+    <hyperlink ref="K30" location="TC_28!A1" display="TC_28!A1"/>
+    <hyperlink ref="K31" location="TC_29!A1" display="TC_29!A1"/>
+    <hyperlink ref="K21" location="TC_19!A1" display="TC_19!A1"/>
+    <hyperlink ref="K22" location="TC_20!A1" display="TC_20!A1"/>
+    <hyperlink ref="K23" location="TC_21!A1" display="TC_21!A1"/>
+    <hyperlink ref="K24" location="TC_22!A1" display="TC_22!A1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -2872,6 +3969,28 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
@@ -2880,21 +3999,180 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>122</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="2:2">
       <c r="B3" t="s">
-        <v>123</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" t="s">
-        <v>124</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2908,23 +4186,74 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>125</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="2:2">
       <c r="B3" t="s">
-        <v>123</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" t="s">
-        <v>124</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -2936,17 +4265,17 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>126</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3" spans="2:2">
       <c r="B3" t="s">
-        <v>123</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" t="s">
-        <v>124</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -2964,7 +4293,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -2982,7 +4311,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>128</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -3000,7 +4329,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>129</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3018,7 +4347,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>130</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -3036,7 +4365,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>131</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>